<commit_message>
docs: handle setup photos in New-Outlet-Setup workbook
Address the images gap: setup needs photographs that a spreadsheet can't
hold. Add a green photo-reference column carrying a file-name/link per row,
supplied alongside the sheet in a shared folder:
- Pumps: sample totalizer-slip photo (-> pumps.slip_artifact_id), required to
  enable slip scanning; serial/model now marked OCR-filled-from-photo.
- Tanks: opening gauge/ATG (Pinelabs) screen photo (-> station_artifacts).
Add an 'Images & photos' section + green legend entry to the README
explaining what photos are needed and how to provide them.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CKmTPEKJVM3Douvg7WSWsx
</commit_message>
<xml_diff>
--- a/docs/New-Outlet-Setup.xlsx
+++ b/docs/New-Outlet-Setup.xlsx
@@ -30,7 +30,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +70,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00548235"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="15"/>
     </font>
@@ -92,7 +98,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -107,6 +113,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,6 +138,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF1FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -156,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -173,17 +189,26 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -191,25 +216,34 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -426,7 +460,7 @@
   <commentList>
     <comment ref="A4" authorId="0" shapeId="0">
       <text>
-        <t>Must match a company on tab 10.</t>
+        <t>Must match a company on tab 11.</t>
       </text>
     </comment>
     <comment ref="C4" authorId="0" shapeId="0">
@@ -654,6 +688,11 @@
         <t>e.g. petrol ≈ 0.735, diesel ≈ 0.825. Optional but recommended.</t>
       </text>
     </comment>
+    <comment ref="F4" authorId="0" shapeId="0">
+      <text>
+        <t>Photo of the gauge / ATG (Pinelabs) screen showing this tank's opening stock at go-live. Put the file name (e.g. Tank-1-gauge.jpg) or a link here; the picture goes in the shared folder. Recommended.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -671,12 +710,17 @@
     </comment>
     <comment ref="B4" authorId="0" shapeId="0">
       <text>
-        <t>Serial printed on the totalizer slip. Unique per live pump.</t>
+        <t>REQUIRED for slip scanning. A photo of the slip this dispenser (Pinelabs / totalizer) prints. Setup OCRs it to read the SERIAL, MODEL and nozzle lines, and keeps it as the reference print-format. Put the file name (e.g. Pump-1-slip.jpg) or a link here; the picture goes in the shared folder.</t>
       </text>
     </comment>
     <comment ref="C4" authorId="0" shapeId="0">
       <text>
-        <t>Make / model of the dispenser.</t>
+        <t>OCR reads this from the slip photo — leave blank if the photo is clear. The owner confirms it before it saves.</t>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="0" shapeId="0">
+      <text>
+        <t>OCR reads this from the slip photo too. Leave blank if the photo is clear.</t>
       </text>
     </comment>
   </commentList>
@@ -691,7 +735,7 @@
   <commentList>
     <comment ref="A4" authorId="0" shapeId="0">
       <text>
-        <t>Label printed on the nozzle, e.g. 1, 2, 3A. Unique within the outlet.</t>
+        <t>Label printed on the nozzle, e.g. 1, 2, 3A. Convention '1.1' = pump1.nozzle1.</t>
       </text>
     </comment>
     <comment ref="B4" authorId="0" shapeId="0">
@@ -706,7 +750,7 @@
     </comment>
     <comment ref="D4" authorId="0" shapeId="0">
       <text>
-        <t>OPTIONAL. The physical dispenser this nozzle sits on.</t>
+        <t>OPTIONAL. Which dispenser (tab 7) this nozzle sits on.</t>
       </text>
     </comment>
     <comment ref="E4" authorId="0" shapeId="0">
@@ -1027,7 +1071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D33"/>
+  <dimension ref="B2:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1043,10 +1087,10 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="26" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>One workbook to stand up a brand-new outlet and all of its setup. Fill the yellow cells; work the tabs top to bottom.</t>
+          <t>One workbook to stand up a brand-new outlet and all of its setup. Fill the yellow cells; work the tabs top to bottom. Photos go in a shared folder — see 'Images &amp; photos' below.</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1169,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Underground tanks: number, fuel, capacity, opening stock, density.</t>
+          <t>Underground tanks: number, fuel, capacity, opening stock, density + opening gauge/ATG photo.</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1181,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>OPTIONAL — the dispenser machines (only if totalizer-slip scanning is used).</t>
+          <t>The dispenser machines + their SAMPLE TOTALIZER-SLIP PHOTO (required for slip scanning).</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1193,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Each nozzle mapped to its tank + fuel (and optionally its dispenser/slip line).</t>
+          <t>Each nozzle mapped to its tank + fuel (and optionally its dispenser / slip line).</t>
         </is>
       </c>
     </row>
@@ -1214,151 +1258,233 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Images &amp; photos  (READ THIS)</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21" ht="44" customHeight="1">
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Some of the setup CANNOT be done from text alone — it needs photographs. A spreadsheet can't hold images, so the sheet holds a FILE-NAME (or a link) per photo and you supply the actual pictures alongside it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1">
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>How: put every photo in ONE shared folder (Google Drive / OneDrive) and name each file after its row — e.g. 'Pump-1-slip.jpg', 'Tank-1-gauge.jpg'. Type that file name (or a direct link) into the green photo column. Then share the folder link with us.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="44" customHeight="1">
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Pump sample slip (green column on tab 7) — REQUIRED for slip scanning. A photo of the totalizer slip the dispenser prints. Setup runs OCR on it to read the pump SERIAL, MODEL and which line is which nozzle, and keeps it as the reference print-format for every future settlement scan. Leave Serial/Model blank if the photo is clear — OCR fills them, and the owner confirms before it's saved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="44" customHeight="1">
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Tank gauge / ATG (Pinelabs) screen (green column on tab 6) — recommended at go-live. A photo of the gauge screen showing opening stock; it's the picture behind the first wet-stock figure the outlet is measured against.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="44" customHeight="1">
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Nozzle meter photos are NOT a setup item — those are captured per shift during settlement, in the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="B21" s="7" t="inlineStr"/>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="11" t="inlineStr"/>
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>Yellow cell — A value YOU fill in.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="B22" s="9" t="inlineStr"/>
-      <c r="C22" s="8" t="inlineStr">
+    <row r="29" ht="20" customHeight="1">
+      <c r="B29" s="13" t="inlineStr"/>
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>Blue header (white text) — REQUIRED column — the row is rejected without it.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="B23" s="10" t="inlineStr"/>
-      <c r="C23" s="8" t="inlineStr">
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="14" t="inlineStr"/>
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>Grey header (white text) — Optional column — safe to leave blank; a sensible default applies.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="B24" s="11" t="inlineStr"/>
-      <c r="C24" s="8" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="15" t="inlineStr"/>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Green header + green cell — A PHOTO reference — put the file name / link here; the picture goes in the shared folder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="B32" s="16" t="inlineStr"/>
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>Italic grey row — An EXAMPLE row showing the expected format. Delete it before import.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="3" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>House rules</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
-      <c r="B27" s="12" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr"/>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="B35" s="17" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C35" s="9" t="inlineStr">
         <is>
           <t>Mobile numbers: 10 Indian digits (e.g. 9876543210). +91 is added automatically. A phone is a login ID — it must be unique.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="B28" s="12" t="inlineStr">
+    <row r="36" ht="28" customHeight="1">
+      <c r="B36" s="17" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>Dates: DD-MMM-YYYY (e.g. 05-Aug-2026). India is DD/MM — never MM/DD.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="28" customHeight="1">
-      <c r="B29" s="12" t="inlineStr">
+    <row r="37" ht="28" customHeight="1">
+      <c r="B37" s="17" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C29" s="13" t="inlineStr">
+      <c r="C37" s="9" t="inlineStr">
         <is>
           <t>Times: 24-hour HH:MM (e.g. 06:00, 14:00, 22:00).</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="B30" s="12" t="inlineStr">
+    <row r="38" ht="28" customHeight="1">
+      <c r="B38" s="17" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C30" s="13" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>Fuel types must be one of: petrol, diesel, premium_petrol, cng, xp95, speed, power. Use the SAME spelling on Tanks, Nozzles and Fuel Prices.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="B31" s="12" t="inlineStr">
+    <row r="39" ht="28" customHeight="1">
+      <c r="B39" s="17" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C31" s="13" t="inlineStr">
+      <c r="C39" s="9" t="inlineStr">
         <is>
           <t>New staff/owners get the starter password 'Welcome@123' and are forced to reset on first login — leave the password blank to use it.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="B32" s="12" t="inlineStr">
+    <row r="40" ht="28" customHeight="1">
+      <c r="B40" s="17" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C32" s="13" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>Money is in ₹. Opening stock is in litres. Density is kg/L (e.g. petrol ≈ 0.735, diesel ≈ 0.825).</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="B33" s="12" t="inlineStr">
+    <row r="41" ht="28" customHeight="1">
+      <c r="B41" s="17" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="C33" s="13" t="inlineStr">
-        <is>
-          <t>This sheet COLLECTS the data; a superadmin runs the actual go-live import. Nothing here writes to production by itself.</t>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>This sheet COLLECTS the data + photo references; a superadmin runs the actual go-live. Nothing here writes to production by itself.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="18">
     <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C34:D34"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C25:D25"/>
     <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C39:D39"/>
     <mergeCell ref="B2:D2"/>
+    <mergeCell ref="C35:D35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1378,27 +1504,27 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>9 · Opening Fuel Prices</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>The per-litre selling price of each fuel at go-live. One row per fuel type the outlet sells. Prices are updated daily in-app after go-live; this just seeds the first price.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Fuel type
 (fuel_prices.fuel_type)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Price ₹/L
 (fuel_prices.price)</t>
@@ -1406,46 +1532,46 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>petrol</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="22" t="n">
         <v>105.5</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1453,7 +1579,7 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="A6:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list (or type a custom one is NOT allowed here)." type="list">
+    <dataValidation sqref="A6:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list." type="list">
       <formula1>"petrol,diesel,premium_petrol,cng,xp95,speed,power"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1478,39 +1604,39 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>10 · Shift Timings</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>The daily shift windows this outlet runs (1 to 3 shifts). Times are 24-hour HH:MM. A shift that crosses midnight is fine (e.g. 22:00 → 06:00).</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Shift #
 (shift_number)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Name
 (shift_definitions.name)</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>Start time
 (start_time)</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>End time
 (end_time)</t>
@@ -1518,42 +1644,42 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="n">
+      <c r="A5" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Morning</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>06:00</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1561,7 +1687,7 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="A6:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list (or type a custom one is NOT allowed here)." type="list">
+    <dataValidation sqref="A6:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list." type="list">
       <formula1>"1,2,3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1587,45 +1713,45 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>11 · Credit (Corporate) Customers</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Corporate / credit accounts that fuel on account. 'Opening balance' is the receivable outstanding at go-live (an opening invoice is raised for it). Dedupe is on mobile within the outlet.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Company name
 (corporate_accounts.company_name)</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Contact mobile
 (contact_phone)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Opening balance ₹
 (→ opening invoice)</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Credit limit ₹
 (corporate_station_links.credit_limit)</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>GSTIN
 (corporate_accounts.gstn)</t>
@@ -1633,139 +1759,139 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>ABC Logistics Pvt Ltd</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>9876543210</t>
         </is>
       </c>
-      <c r="C5" s="18" t="n">
+      <c r="C5" s="22" t="n">
         <v>45000</v>
       </c>
-      <c r="D5" s="18" t="n">
+      <c r="D5" s="22" t="n">
         <v>200000</v>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>36ABCDE1234F1Z5</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="n"/>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n"/>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
+      <c r="A21" s="11" t="n"/>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1797,63 +1923,63 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>12 · Products  (OPTIONAL — only if the store module is used)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Shop / lubricant products sold at the outlet's store. Skip this tab entirely if the outlet only sells fuel.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Product name
 (products.name)</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Brand
 (products.brand)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Unit
 (products.unit)</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>Selling price ₹
 (selling_price)</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>Buying price ₹
 (buying_price)</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>GST %
 (gst_rate)</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="G4" s="21" t="inlineStr">
         <is>
           <t>HSN code
 (hsn_code)</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="H4" s="21" t="inlineStr">
         <is>
           <t>Opening stock
 (current_stock)</t>
@@ -1861,178 +1987,178 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Servo 4T 900ml</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Servo</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>piece</t>
         </is>
       </c>
-      <c r="D5" s="18" t="n">
+      <c r="D5" s="22" t="n">
         <v>480</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="22" t="n">
         <v>360</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="22" t="n">
         <v>18</v>
       </c>
-      <c r="G5" s="18" t="inlineStr">
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>27101980</t>
         </is>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="22" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="11" t="n"/>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="7" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="n"/>
-      <c r="H12" s="7" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="7" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
-      <c r="H14" s="7" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
+      <c r="H14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
-      <c r="G15" s="7" t="n"/>
-      <c r="H15" s="7" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
+      <c r="H15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="7" t="n"/>
-      <c r="G16" s="7" t="n"/>
-      <c r="H16" s="7" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
+      <c r="H16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="7" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
-      <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="7" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="11" t="n"/>
+      <c r="H19" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2062,51 +2188,51 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>13 · Corporate Drivers / Vehicles  (OPTIONAL)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Drivers and vehicles under a credit customer — used by RFID / FastTag fleet fuelling. The 'Company name' must match a row on the Credit Customers tab.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Company name
 (→ Credit Customers)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Driver name
 (corporate_drivers.name)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Driver mobile
 (phone)</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Vehicle number
 (vehicle_number)</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>FastTag / RFID id
 (fasttag_id)</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>Per-fill limit ₹
 (per_fill_limit)</t>
@@ -2114,146 +2240,146 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>ABC Logistics Pvt Ltd</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Rajan M</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>9876000001</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>TS09AB1234</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>FT123456</t>
         </is>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="22" t="n">
         <v>5000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="7" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="7" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
-      <c r="F19" s="7" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2283,51 +2409,51 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>1 · Owner &amp; Owner Group</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>The owner group is the billing entity that can hold several outlets; the owner is the top login. Create these first — the outlet is attached to them. One row each.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Owner Group name
 (owner_groups.name)</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Group description
 (owner_groups.description)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Billing email
 (subscriptions.billing_email)</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>Owner name
 (users.name)</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>Owner mobile
 (users.phone)</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>Owner email
 (users.email)</t>
@@ -2335,84 +2461,84 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Kamala Fuels</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Kamala group of outlets</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>billing@kamala.in</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>Ramesh Kamala</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>9876500001</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>ramesh@kamala.in</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2460,159 +2586,159 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>2 · Outlet (station + settings)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>The station and all of its settings on ONE row. Blue = required to create the outlet; the rest are station settings with sensible defaults if left blank.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Outlet name
 (stations.name)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Oil company
 (stations.oil_company)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Address
 (stations.address)</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>City
 (stations.city)</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>State
 (stations.state)</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>Pincode
 (station_settings.pincode)</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="G4" s="21" t="inlineStr">
         <is>
           <t>GSTIN
 (gst_number / gstn)</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="H4" s="21" t="inlineStr">
         <is>
           <t>PAN
 (station_settings.pan)</t>
         </is>
       </c>
-      <c r="I4" s="17" t="inlineStr">
+      <c r="I4" s="21" t="inlineStr">
         <is>
           <t>TAN
 (station_settings.tan)</t>
         </is>
       </c>
-      <c r="J4" s="17" t="inlineStr">
+      <c r="J4" s="21" t="inlineStr">
         <is>
           <t>Owner WhatsApp
 (owner_whatsapp)</t>
         </is>
       </c>
-      <c r="K4" s="17" t="inlineStr">
+      <c r="K4" s="21" t="inlineStr">
         <is>
           <t>Owner email
 (station_settings.owner_email)</t>
         </is>
       </c>
-      <c r="L4" s="17" t="inlineStr">
+      <c r="L4" s="21" t="inlineStr">
         <is>
           <t>Language
 (language)</t>
         </is>
       </c>
-      <c r="M4" s="17" t="inlineStr">
+      <c r="M4" s="21" t="inlineStr">
         <is>
           <t>Invoice prefix
 (invoice_prefix)</t>
         </is>
       </c>
-      <c r="N4" s="17" t="inlineStr">
+      <c r="N4" s="21" t="inlineStr">
         <is>
           <t>Variance threshold ₹
 (variance_threshold)</t>
         </is>
       </c>
-      <c r="O4" s="17" t="inlineStr">
+      <c r="O4" s="21" t="inlineStr">
         <is>
           <t>Latitude
 (latitude)</t>
         </is>
       </c>
-      <c r="P4" s="17" t="inlineStr">
+      <c r="P4" s="21" t="inlineStr">
         <is>
           <t>Longitude
 (longitude)</t>
         </is>
       </c>
-      <c r="Q4" s="17" t="inlineStr">
+      <c r="Q4" s="21" t="inlineStr">
         <is>
           <t>Geofence radius m
 (geo_fence_radius)</t>
         </is>
       </c>
-      <c r="R4" s="17" t="inlineStr">
+      <c r="R4" s="21" t="inlineStr">
         <is>
           <t>Geofence on?
 (geo_fence_enabled)</t>
         </is>
       </c>
-      <c r="S4" s="17" t="inlineStr">
+      <c r="S4" s="21" t="inlineStr">
         <is>
           <t>Manager blind-drop?
 (manager_blind_drop)</t>
         </is>
       </c>
-      <c r="T4" s="17" t="inlineStr">
+      <c r="T4" s="21" t="inlineStr">
         <is>
           <t>Stock tol % petrol
 (stock_tol_pct_petrol)</t>
         </is>
       </c>
-      <c r="U4" s="17" t="inlineStr">
+      <c r="U4" s="21" t="inlineStr">
         <is>
           <t>Stock tol % diesel
 (stock_tol_pct_diesel)</t>
         </is>
       </c>
-      <c r="V4" s="17" t="inlineStr">
+      <c r="V4" s="21" t="inlineStr">
         <is>
           <t>Stock tol floor L
 (stock_tol_floor_ltrs)</t>
         </is>
       </c>
-      <c r="W4" s="17" t="inlineStr">
+      <c r="W4" s="21" t="inlineStr">
         <is>
           <t>Deposit alert days
 (deposit_alert_days)</t>
         </is>
       </c>
-      <c r="X4" s="17" t="inlineStr">
+      <c r="X4" s="21" t="inlineStr">
         <is>
           <t>Tally company
 (tally_company_name)</t>
@@ -2620,218 +2746,218 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Kamala Highway</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>HPCL</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>NH-44, Kompally</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>Hyderabad</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>Telangana</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>500014</t>
         </is>
       </c>
-      <c r="G5" s="18" t="inlineStr">
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>36ABCDE1234F1Z5</t>
         </is>
       </c>
-      <c r="H5" s="18" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>ABCDE1234F</t>
         </is>
       </c>
-      <c r="I5" s="18" t="inlineStr">
+      <c r="I5" s="22" t="inlineStr">
         <is>
           <t>HYDK12345A</t>
         </is>
       </c>
-      <c r="J5" s="18" t="inlineStr">
+      <c r="J5" s="22" t="inlineStr">
         <is>
           <t>9876500001</t>
         </is>
       </c>
-      <c r="K5" s="18" t="inlineStr">
+      <c r="K5" s="22" t="inlineStr">
         <is>
           <t>owner@kamala.in</t>
         </is>
       </c>
-      <c r="L5" s="18" t="inlineStr">
+      <c r="L5" s="22" t="inlineStr">
         <is>
           <t>en</t>
         </is>
       </c>
-      <c r="M5" s="18" t="inlineStr">
+      <c r="M5" s="22" t="inlineStr">
         <is>
           <t>KAM</t>
         </is>
       </c>
-      <c r="N5" s="18" t="n">
+      <c r="N5" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="O5" s="18" t="inlineStr">
+      <c r="O5" s="22" t="inlineStr">
         <is>
           <t>17.5810</t>
         </is>
       </c>
-      <c r="P5" s="18" t="inlineStr">
+      <c r="P5" s="22" t="inlineStr">
         <is>
           <t>78.4990</t>
         </is>
       </c>
-      <c r="Q5" s="18" t="n">
+      <c r="Q5" s="22" t="n">
         <v>500</v>
       </c>
-      <c r="R5" s="18" t="inlineStr">
+      <c r="R5" s="22" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="S5" s="18" t="inlineStr">
+      <c r="S5" s="22" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="T5" s="18" t="n">
+      <c r="T5" s="22" t="n">
         <v>0.75</v>
       </c>
-      <c r="U5" s="18" t="n">
+      <c r="U5" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="V5" s="18" t="n">
+      <c r="V5" s="22" t="n">
         <v>20</v>
       </c>
-      <c r="W5" s="18" t="n">
+      <c r="W5" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="X5" s="18" t="inlineStr">
+      <c r="X5" s="22" t="inlineStr">
         <is>
           <t>Kamala Highway HPCL</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
-      <c r="M6" s="7" t="n"/>
-      <c r="N6" s="7" t="n"/>
-      <c r="O6" s="7" t="n"/>
-      <c r="P6" s="7" t="n"/>
-      <c r="Q6" s="7" t="n"/>
-      <c r="R6" s="7" t="n"/>
-      <c r="S6" s="7" t="n"/>
-      <c r="T6" s="7" t="n"/>
-      <c r="U6" s="7" t="n"/>
-      <c r="V6" s="7" t="n"/>
-      <c r="W6" s="7" t="n"/>
-      <c r="X6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="11" t="n"/>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="11" t="n"/>
+      <c r="I6" s="11" t="n"/>
+      <c r="J6" s="11" t="n"/>
+      <c r="K6" s="11" t="n"/>
+      <c r="L6" s="11" t="n"/>
+      <c r="M6" s="11" t="n"/>
+      <c r="N6" s="11" t="n"/>
+      <c r="O6" s="11" t="n"/>
+      <c r="P6" s="11" t="n"/>
+      <c r="Q6" s="11" t="n"/>
+      <c r="R6" s="11" t="n"/>
+      <c r="S6" s="11" t="n"/>
+      <c r="T6" s="11" t="n"/>
+      <c r="U6" s="11" t="n"/>
+      <c r="V6" s="11" t="n"/>
+      <c r="W6" s="11" t="n"/>
+      <c r="X6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
-      <c r="O7" s="7" t="n"/>
-      <c r="P7" s="7" t="n"/>
-      <c r="Q7" s="7" t="n"/>
-      <c r="R7" s="7" t="n"/>
-      <c r="S7" s="7" t="n"/>
-      <c r="T7" s="7" t="n"/>
-      <c r="U7" s="7" t="n"/>
-      <c r="V7" s="7" t="n"/>
-      <c r="W7" s="7" t="n"/>
-      <c r="X7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="11" t="n"/>
+      <c r="I7" s="11" t="n"/>
+      <c r="J7" s="11" t="n"/>
+      <c r="K7" s="11" t="n"/>
+      <c r="L7" s="11" t="n"/>
+      <c r="M7" s="11" t="n"/>
+      <c r="N7" s="11" t="n"/>
+      <c r="O7" s="11" t="n"/>
+      <c r="P7" s="11" t="n"/>
+      <c r="Q7" s="11" t="n"/>
+      <c r="R7" s="11" t="n"/>
+      <c r="S7" s="11" t="n"/>
+      <c r="T7" s="11" t="n"/>
+      <c r="U7" s="11" t="n"/>
+      <c r="V7" s="11" t="n"/>
+      <c r="W7" s="11" t="n"/>
+      <c r="X7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
-      <c r="O8" s="7" t="n"/>
-      <c r="P8" s="7" t="n"/>
-      <c r="Q8" s="7" t="n"/>
-      <c r="R8" s="7" t="n"/>
-      <c r="S8" s="7" t="n"/>
-      <c r="T8" s="7" t="n"/>
-      <c r="U8" s="7" t="n"/>
-      <c r="V8" s="7" t="n"/>
-      <c r="W8" s="7" t="n"/>
-      <c r="X8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="11" t="n"/>
+      <c r="I8" s="11" t="n"/>
+      <c r="J8" s="11" t="n"/>
+      <c r="K8" s="11" t="n"/>
+      <c r="L8" s="11" t="n"/>
+      <c r="M8" s="11" t="n"/>
+      <c r="N8" s="11" t="n"/>
+      <c r="O8" s="11" t="n"/>
+      <c r="P8" s="11" t="n"/>
+      <c r="Q8" s="11" t="n"/>
+      <c r="R8" s="11" t="n"/>
+      <c r="S8" s="11" t="n"/>
+      <c r="T8" s="11" t="n"/>
+      <c r="U8" s="11" t="n"/>
+      <c r="V8" s="11" t="n"/>
+      <c r="W8" s="11" t="n"/>
+      <c r="X8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
-      <c r="O9" s="7" t="n"/>
-      <c r="P9" s="7" t="n"/>
-      <c r="Q9" s="7" t="n"/>
-      <c r="R9" s="7" t="n"/>
-      <c r="S9" s="7" t="n"/>
-      <c r="T9" s="7" t="n"/>
-      <c r="U9" s="7" t="n"/>
-      <c r="V9" s="7" t="n"/>
-      <c r="W9" s="7" t="n"/>
-      <c r="X9" s="7" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="11" t="n"/>
+      <c r="I9" s="11" t="n"/>
+      <c r="J9" s="11" t="n"/>
+      <c r="K9" s="11" t="n"/>
+      <c r="L9" s="11" t="n"/>
+      <c r="M9" s="11" t="n"/>
+      <c r="N9" s="11" t="n"/>
+      <c r="O9" s="11" t="n"/>
+      <c r="P9" s="11" t="n"/>
+      <c r="Q9" s="11" t="n"/>
+      <c r="R9" s="11" t="n"/>
+      <c r="S9" s="11" t="n"/>
+      <c r="T9" s="11" t="n"/>
+      <c r="U9" s="11" t="n"/>
+      <c r="V9" s="11" t="n"/>
+      <c r="W9" s="11" t="n"/>
+      <c r="X9" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2839,13 +2965,13 @@
     <mergeCell ref="A1:X1"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation sqref="L6:L200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list (or type a custom one is NOT allowed here)." type="list">
+    <dataValidation sqref="L6:L200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list." type="list">
       <formula1>"en,te,ta,hi"</formula1>
     </dataValidation>
-    <dataValidation sqref="R6:R200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list (or type a custom one is NOT allowed here)." type="list">
+    <dataValidation sqref="R6:R200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list." type="list">
       <formula1>"yes,no"</formula1>
     </dataValidation>
-    <dataValidation sqref="S6:S200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list (or type a custom one is NOT allowed here)." type="list">
+    <dataValidation sqref="S6:S200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list." type="list">
       <formula1>"yes,no"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2870,39 +2996,39 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>3 · Subscription / Plan</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>The plan this outlet runs on. The plan drives the feature ceiling (entitlement): a plan whose name contains 'lite' → the Lite feature set, otherwise the full Pumpini set. One row.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Plan
 (station_subscriptions.plan)</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Status
 (status)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Start date
 (start_date)</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>End date
 (end_date)</t>
@@ -2910,40 +3036,40 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>pro</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>05-Aug-2026</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr"/>
+      <c r="D5" s="22" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2951,10 +3077,10 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="A6:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list (or type a custom one is NOT allowed here)." type="list">
+    <dataValidation sqref="A6:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list." type="list">
       <formula1>"pro,lite,trial"</formula1>
     </dataValidation>
-    <dataValidation sqref="B6:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list (or type a custom one is NOT allowed here)." type="list">
+    <dataValidation sqref="B6:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list." type="list">
       <formula1>"active,suspended,cancelled"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2980,45 +3106,45 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>4 · Managers &amp; Back-office (CCO)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Managers run the outlet day-to-day; CCO (Central Cash Office) users get back-office access across the owner group. Attendants go on the next tab. Leave password blank to use the 'Welcome@123' starter.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Name
 (users.name)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Mobile
 (users.phone)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Email
 (users.email)</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>Role
 (users.role)</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>Starter password
 (password)</t>
@@ -3026,97 +3152,97 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Suresh Manager</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>9876500010</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>suresh@kamala.in</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>manager</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr"/>
+      <c r="E5" s="22" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3124,7 +3250,7 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="D6:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list (or type a custom one is NOT allowed here)." type="list">
+    <dataValidation sqref="D6:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list." type="list">
       <formula1>"manager,cco"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3148,33 +3274,33 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>5 · Attendants (operators)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>The operators who run the nozzles and settle shifts. Name + mobile is all that is required; they get 'Welcome@123' and reset on first login. An existing number is re-activated, not duplicated.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Name
 (users.name)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Mobile
 (users.phone)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Language
 (users.language)</t>
@@ -3182,121 +3308,121 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Arjun S</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>9876500020</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>te</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="n"/>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n"/>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="n"/>
+      <c r="A21" s="11" t="n"/>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="n"/>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="11" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="n"/>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="n"/>
+      <c r="A23" s="11" t="n"/>
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="11" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="n"/>
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="7" t="n"/>
+      <c r="A24" s="11" t="n"/>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="n"/>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="7" t="n"/>
+      <c r="A25" s="11" t="n"/>
+      <c r="B25" s="11" t="n"/>
+      <c r="C25" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3304,7 +3430,7 @@
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C6:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list (or type a custom one is NOT allowed here)." type="list">
+    <dataValidation sqref="C6:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list." type="list">
       <formula1>"en,te,ta,hi"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3319,7 +3445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3327,164 +3453,188 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>6 · Tanks</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
-        <is>
-          <t>One row per underground tank. 'Opening stock' is the dip-verified stock at go-live. Tank number is referenced by nozzles on the next tab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>One row per underground tank. 'Opening stock' is the dip-verified stock at go-live. Tank number is referenced by nozzles on tab 8. The green column is the file name / link of the opening gauge photo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Tank #
 (tanks.tank_number)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Fuel type
 (tanks.fuel_type)</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>Capacity L
 (capacity_ltrs)</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>Opening stock L
 (current_stock)</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>Density kg/L
 (density)</t>
         </is>
       </c>
+      <c r="F4" s="23" t="inlineStr">
+        <is>
+          <t>Opening gauge/ATG photo
+(file name / link → station_artifacts)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="n">
+      <c r="A5" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>petrol</t>
         </is>
       </c>
-      <c r="C5" s="18" t="n">
+      <c r="C5" s="22" t="n">
         <v>20000</v>
       </c>
-      <c r="D5" s="18" t="n">
+      <c r="D5" s="22" t="n">
         <v>15000</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="22" t="n">
         <v>0.735</v>
       </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>Tank-1-gauge.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="24" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="24" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="24" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="24" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="24" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="24" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="24" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="24" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="24" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="24" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="24" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B6:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list (or type a custom one is NOT allowed here)." type="list">
+    <dataValidation sqref="B6:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list." type="list">
       <formula1>"petrol,diesel,premium_petrol,cng,xp95,speed,power"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3499,49 +3649,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
-          <t>7 · Pumps / Dispensers  (OPTIONAL)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
-        <is>
-          <t>The physical dispenser machines. A pump is a MACHINE, not a fuel — several nozzles (grades) sit on it. Only needed if the outlet scans totalizer slips; otherwise skip and leave the pump columns blank on Nozzles.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>7 · Pumps / Dispensers  (+ sample slip photo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>The physical dispenser machines. A pump is a MACHINE, not a fuel — several nozzles (grades) sit on it. The green column is the SAMPLE TOTALIZER-SLIP PHOTO — required to enable slip scanning at settlement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Pump no
 (pumps.pump_number)</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>Sample totalizer-slip photo
+(file name / link → pumps.slip_artifact_id)</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Serial
 (pumps.serial)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Model
 (pumps.model)</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>Notes
 (pumps.notes)</t>
@@ -3549,91 +3706,98 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>GVR-9823-A</t>
-        </is>
-      </c>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>Gilbarco SK700</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Front island</t>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>Pump-1-slip.jpg</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr"/>
+      <c r="D5" s="22" t="inlineStr"/>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>Front island — OCR fills serial/model</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="24" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="24" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="24" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="24" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="24" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="24" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="24" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="24" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="24" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -3652,50 +3816,50 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>8 · Nozzles</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
-        <is>
-          <t>One row per nozzle. Each nozzle belongs to a tank (match the Tank # from the Tanks tab) and dispenses that tank's fuel. Dispenser / slip-line columns are optional (only if totalizer-slip scanning is used).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>One row per nozzle. Each nozzle belongs to a tank (match the Tank # from the Tanks tab) and dispenses that tank's fuel. Pump no + slip line are optional (only if totalizer-slip scanning is used).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Nozzle #
 (nozzles.nozzle_number)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Tank #
 (→ tanks.tank_number)</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>Fuel type
 (nozzles.fuel_type)</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
-        <is>
-          <t>Dispenser / pump no
-(pump_id → pumps)</t>
-        </is>
-      </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>Pump no
+(→ pumps.pump_number)</t>
+        </is>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>Slip line no
 (slip_nozzle_no)</t>
@@ -3703,137 +3867,139 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="n">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>petrol</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>petrol</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>DU-1</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="n"/>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n"/>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
+      <c r="A21" s="11" t="n"/>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3841,7 +4007,7 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C6:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list (or type a custom one is NOT allowed here)." type="list">
+    <dataValidation sqref="C6:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list." type="list">
       <formula1>"petrol,diesel,premium_petrol,cng,xp95,speed,power"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs: add Credit Slip Books (booklet allocation + slip format) tab
Missing from onboarding: credit customers are issued pre-printed coupon
booklets and each booklet's slip format needs to be on record.

- New tab 12 'Credit Slip Books' -> credit_slip_books: company (corporate_id),
  book_label, series_start/end, opening_leaf, issued_on, status, with the
  no-overlap series range that catches a missing/re-used coupon.
- Green 'Sample coupon photo' column captures the slip format the coupon
  parser reads. (No dedicated per-customer format store exists yet; captured
  as a reference pending a backend home.)
- Renumber Products -> 13, Corporate Drivers -> 14; README order + Images
  section updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CKmTPEKJVM3Douvg7WSWsx
</commit_message>
<xml_diff>
--- a/docs/New-Outlet-Setup.xlsx
+++ b/docs/New-Outlet-Setup.xlsx
@@ -19,8 +19,9 @@
     <sheet name="9. Fuel Prices" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="10. Shift Timings" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="11. Credit Customers" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="12. Products" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="13. Corporate Drivers" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="12. Credit Slip Books" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="13. Products" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="14. Corporate Drivers" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,19 +434,44 @@
     <author>Pumpini</author>
   </authors>
   <commentList>
+    <comment ref="A4" authorId="0" shapeId="0">
+      <text>
+        <t>Which credit customer this booklet is issued to. Must match a company on tab 11.</t>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>Optional printed book id / name. Free text.</t>
+      </text>
+    </comment>
     <comment ref="C4" authorId="0" shapeId="0">
       <text>
-        <t>piece / litre / kg. Default piece.</t>
+        <t>The FIRST coupon number in the book, e.g. 17701. Ranges must not overlap another book at this outlet.</t>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="0" shapeId="0">
+      <text>
+        <t>The LAST coupon number in the book, e.g. 17800. Must be ≥ series start.</t>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="0" shapeId="0">
+      <text>
+        <t>Only if the book is handed over PART-USED — the first still-blank coupon. Blank = starts at series start.</t>
       </text>
     </comment>
     <comment ref="F4" authorId="0" shapeId="0">
       <text>
-        <t>Default 18.</t>
+        <t>Date the book was handed over. Default = today.</t>
+      </text>
+    </comment>
+    <comment ref="G4" authorId="0" shapeId="0">
+      <text>
+        <t>active / exhausted / cancelled / lost. Default active.</t>
       </text>
     </comment>
     <comment ref="H4" authorId="0" shapeId="0">
       <text>
-        <t>Units in stock at go-live.</t>
+        <t>One photo of a coupon from THIS booklet — records the slip format the parser reads (Coupon No, Date, Vehicle, litres, seal). Put the file name (e.g. Coupon-ABC-sample.jpg) or a link here; picture goes in the shared folder. Note: there is no dedicated store for a per-customer format sample yet — see the chat note.</t>
       </text>
     </comment>
   </commentList>
@@ -453,6 +479,31 @@
 </file>
 
 <file path=xl/comments/comment13.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Pumpini</author>
+  </authors>
+  <commentList>
+    <comment ref="C4" authorId="0" shapeId="0">
+      <text>
+        <t>piece / litre / kg. Default piece.</t>
+      </text>
+    </comment>
+    <comment ref="F4" authorId="0" shapeId="0">
+      <text>
+        <t>Default 18.</t>
+      </text>
+    </comment>
+    <comment ref="H4" authorId="0" shapeId="0">
+      <text>
+        <t>Units in stock at go-live.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment14.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Pumpini</author>
@@ -1071,7 +1122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D41"/>
+  <dimension ref="B2:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1236,46 +1287,46 @@
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>12. Products</t>
+          <t>12. Credit Slip Books</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>OPTIONAL — shop / lubricant products, only if the outlet uses the store module.</t>
+          <t>Coupon booklets allocated to a credit customer: series range + a sample coupon photo.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>13. Corporate Drivers</t>
+          <t>13. Products</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
+          <t>OPTIONAL — shop / lubricant products, only if the outlet uses the store module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>14. Corporate Drivers</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
           <t>OPTIONAL — drivers/vehicles under a credit customer (RFID/FastTag fleets).</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="6" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Images &amp; photos  (READ THIS)</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr"/>
-    </row>
-    <row r="21" ht="44" customHeight="1">
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Some of the setup CANNOT be done from text alone — it needs photographs. A spreadsheet can't hold images, so the sheet holds a FILE-NAME (or a link) per photo and you supply the actual pictures alongside it.</t>
-        </is>
-      </c>
+      <c r="C21" s="7" t="inlineStr"/>
     </row>
     <row r="22" ht="44" customHeight="1">
       <c r="B22" s="8" t="inlineStr">
@@ -1285,7 +1336,7 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>How: put every photo in ONE shared folder (Google Drive / OneDrive) and name each file after its row — e.g. 'Pump-1-slip.jpg', 'Tank-1-gauge.jpg'. Type that file name (or a direct link) into the green photo column. Then share the folder link with us.</t>
+          <t>Some of the setup CANNOT be done from text alone — it needs photographs. A spreadsheet can't hold images, so the sheet holds a FILE-NAME (or a link) per photo and you supply the actual pictures alongside it.</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1348,7 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Pump sample slip (green column on tab 7) — REQUIRED for slip scanning. A photo of the totalizer slip the dispenser prints. Setup runs OCR on it to read the pump SERIAL, MODEL and which line is which nozzle, and keeps it as the reference print-format for every future settlement scan. Leave Serial/Model blank if the photo is clear — OCR fills them, and the owner confirms before it's saved.</t>
+          <t>How: put every photo in ONE shared folder (Google Drive / OneDrive) and name each file after its row — e.g. 'Pump-1-slip.jpg', 'Tank-1-gauge.jpg'. Type that file name (or a direct link) into the green photo column. Then share the folder link with us.</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1360,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Tank gauge / ATG (Pinelabs) screen (green column on tab 6) — recommended at go-live. A photo of the gauge screen showing opening stock; it's the picture behind the first wet-stock figure the outlet is measured against.</t>
+          <t>Pump sample slip (green column on tab 7) — REQUIRED for slip scanning. A photo of the totalizer slip the dispenser prints. Setup runs OCR on it to read the pump SERIAL, MODEL and which line is which nozzle, and keeps it as the reference print-format for every future settlement scan. Leave Serial/Model blank if the photo is clear — OCR fills them, and the owner confirms before it's saved.</t>
         </is>
       </c>
     </row>
@@ -1321,89 +1372,89 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
+          <t>Tank gauge / ATG (Pinelabs) screen (green column on tab 6) — recommended at go-live. A photo of the gauge screen showing opening stock; it's the picture behind the first wet-stock figure the outlet is measured against.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="44" customHeight="1">
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Credit-coupon sample (green column on tab 12) — one photo per credit customer's booklet. It records the SLIP FORMAT the coupon parser will read (Coupon No, Date, Vehicle, litres, seal). A sample per customer/dealer, not per coupon — the live coupons are photographed per sale in the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="44" customHeight="1">
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
           <t>Nozzle meter photos are NOT a setup item — those are captured per shift during settlement, in the app.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="3" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
-      <c r="C27" s="10" t="inlineStr"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="B28" s="11" t="inlineStr"/>
-      <c r="C28" s="12" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="11" t="inlineStr"/>
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>Yellow cell — A value YOU fill in.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="B29" s="13" t="inlineStr"/>
-      <c r="C29" s="12" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="13" t="inlineStr"/>
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>Blue header (white text) — REQUIRED column — the row is rejected without it.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="14" t="inlineStr"/>
-      <c r="C30" s="12" t="inlineStr">
+    <row r="32" ht="20" customHeight="1">
+      <c r="B32" s="14" t="inlineStr"/>
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>Grey header (white text) — Optional column — safe to leave blank; a sensible default applies.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="B31" s="15" t="inlineStr"/>
-      <c r="C31" s="12" t="inlineStr">
+    <row r="33" ht="20" customHeight="1">
+      <c r="B33" s="15" t="inlineStr"/>
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>Green header + green cell — A PHOTO reference — put the file name / link here; the picture goes in the shared folder.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="B32" s="16" t="inlineStr"/>
-      <c r="C32" s="12" t="inlineStr">
+    <row r="34" ht="20" customHeight="1">
+      <c r="B34" s="16" t="inlineStr"/>
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>Italic grey row — An EXAMPLE row showing the expected format. Delete it before import.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="3" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>House rules</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr"/>
-    </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="B35" s="17" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Mobile numbers: 10 Indian digits (e.g. 9876543210). +91 is added automatically. A phone is a login ID — it must be unique.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="B36" s="17" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>Dates: DD-MMM-YYYY (e.g. 05-Aug-2026). India is DD/MM — never MM/DD.</t>
-        </is>
-      </c>
+      <c r="C36" s="10" t="inlineStr"/>
     </row>
     <row r="37" ht="28" customHeight="1">
       <c r="B37" s="17" t="inlineStr">
@@ -1413,7 +1464,7 @@
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Times: 24-hour HH:MM (e.g. 06:00, 14:00, 22:00).</t>
+          <t>Mobile numbers: 10 Indian digits (e.g. 9876543210). +91 is added automatically. A phone is a login ID — it must be unique.</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1476,7 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Fuel types must be one of: petrol, diesel, premium_petrol, cng, xp95, speed, power. Use the SAME spelling on Tanks, Nozzles and Fuel Prices.</t>
+          <t>Dates: DD-MMM-YYYY (e.g. 05-Aug-2026). India is DD/MM — never MM/DD.</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1488,7 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>New staff/owners get the starter password 'Welcome@123' and are forced to reset on first login — leave the password blank to use it.</t>
+          <t>Times: 24-hour HH:MM (e.g. 06:00, 14:00, 22:00).</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1500,7 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Money is in ₹. Opening stock is in litres. Density is kg/L (e.g. petrol ≈ 0.735, diesel ≈ 0.825).</t>
+          <t>Fuel types must be one of: petrol, diesel, premium_petrol, cng, xp95, speed, power. Use the SAME spelling on Tanks, Nozzles and Fuel Prices.</t>
         </is>
       </c>
     </row>
@@ -1461,30 +1512,55 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
+          <t>New staff/owners get the starter password 'Welcome@123' and are forced to reset on first login — leave the password blank to use it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="B42" s="17" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Money is in ₹. Opening stock is in litres. Density is kg/L (e.g. petrol ≈ 0.735, diesel ≈ 0.825).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="B43" s="17" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
           <t>This sheet COLLECTS the data + photo references; a superadmin runs the actual go-live. Nothing here writes to production by itself.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="B3:D3"/>
+  <mergeCells count="19">
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C43:D43"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="C25:D25"/>
     <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="C37:D37"/>
     <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C40:D40"/>
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="C39:D39"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C37:D37"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="C35:D35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1909,6 +1985,258 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>12 · Credit Slip Books (coupon booklets)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>The pre-printed coupon booklets allocated to a credit customer. One row per booklet. The coupon series range is recorded so a missing / re-used coupon can be caught; the green column holds a sample coupon photo that records the slip format. Company name must match a row on tab 11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Company name
+(→ Credit Customers)</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Book label
+(credit_slip_books.book_label)</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Series start
+(series_start)</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Series end
+(series_end)</t>
+        </is>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>First unused #
+(opening_leaf)</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>Issued on
+(issued_on)</t>
+        </is>
+      </c>
+      <c r="G4" s="21" t="inlineStr">
+        <is>
+          <t>Status
+(status)</t>
+        </is>
+      </c>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>Sample coupon photo
+(slip format → coupon artifact)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>ABC Logistics Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>Book-A/26-27</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>17701</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>17800</v>
+      </c>
+      <c r="E5" s="22" t="inlineStr"/>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>05-Aug-2026</t>
+        </is>
+      </c>
+      <c r="G5" s="22" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>Coupon-ABC-sample.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="11" t="n"/>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="24" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="24" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="24" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="24" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="24" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="24" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="24" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="24" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
+      <c r="H14" s="24" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
+      <c r="H15" s="24" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
+      <c r="H16" s="24" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="24" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="G6:G200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choose from list" error="Pick a value from the list." type="list">
+      <formula1>"active,exhausted,cancelled,lost"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1925,7 +2253,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>12 · Products  (OPTIONAL — only if the store module is used)</t>
+          <t>13 · Products  (OPTIONAL — only if the store module is used)</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2498,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2190,7 +2518,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>13 · Corporate Drivers / Vehicles  (OPTIONAL)</t>
+          <t>14 · Corporate Drivers / Vehicles  (OPTIONAL)</t>
         </is>
       </c>
     </row>

</xml_diff>